<commit_message>
fix: align Xiasha roadshow scoring and data evidence
</commit_message>
<xml_diff>
--- a/data/schemes/方案录入模板.xlsx
+++ b/data/schemes/方案录入模板.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -697,6 +697,28 @@
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>project_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>暂不纳入评分的代理指标</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>本项目暂不纳入评分的代理指标；仅允许 G-05、Q-05、Q-06，不能关闭硬约束。应在案例来源与边界中记录原因、资料依据和核对人；不适用项不参与维度均值。</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>scoring_exclusions</t>
         </is>
       </c>
     </row>

</xml_diff>